<commit_message>
Mise à jour hebdomadaire — 2026-09-14
Reconstitue la fenêtre de collecte en lisant directement les branches
bulletin/AAAA-MM-JJ distantes (jamais fusionnées vers main depuis le
2026-07-21, cf. note ajoutée à bulletins/_a_traiter.md), puis intègre les
trois évolutions franchissant le seuil de crédibilité ≤ 3 STANAG 2511 :
l'incident de Second Thomas Shoal (20-21/07), l'intégration du missile
hypersonique YJ-20 sur destroyer Type-052D (30/07), et le nouveau radar
AESA rotatif du destroyer Weinan (Type-052D, 03/09).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxEQDANfeuu8D9j679tk7i
</commit_message>
<xml_diff>
--- a/documents/Capacites_Militaires_Chinoises_RPC.xlsx
+++ b/documents/Capacites_Militaires_Chinoises_RPC.xlsx
@@ -2059,12 +2059,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Colonne vertébrale de la flotte hauturière, VLS universel 8 cellules, missiles YJ-18A et SAM HHQ-9B.</t>
+          <t>Colonne vertébrale de la flotte hauturière, VLS universel 8 cellules, missiles YJ-18A et SAM HHQ-9B. Mise à jour 2026 : intégration documentée du missile hypersonique antinavire YJ-20 (Mach 6+/10, portée 1 000-1 500 km) sur destroyer Type-052D fin juillet 2026, jusque-là vu uniquement sur Type-055 ; unité récente Weinan (admise au service, exercice du 1-2 septembre 2026) dotée d'un radar biface AESA rotatif remplaçant le dôme radar sphérique des Type-052D antérieurs.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>IISS, The Military Balance 2026, Chapitre 5 Asie - Chine, p.252</t>
+          <t>IISS, The Military Balance 2026, Chapitre 5 Asie - Chine, p.252 ; The War Zone, 30/07/2026 [C2] ; MilitaryWatchMagazine, 30/07/2026 [C3] ; Global Times / MND chinois, 02-03/09/2026 [B2] ; Zona Militar, 03/09/2026 [B2]</t>
         </is>
       </c>
     </row>

</xml_diff>